<commit_message>
feat: complete UniSIRAJ CIA Helpdesk Agent with Cloud Run & GitHub deployment
</commit_message>
<xml_diff>
--- a/backend/app/data/unisiraj_students_master.xlsx
+++ b/backend/app/data/unisiraj_students_master.xlsx
@@ -447,16 +447,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
     <col width="47" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -582,45 +582,49 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 10:28 UTC</t>
+          <t>2026-10-22 14:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>8231123010</t>
+          <t>11111111111</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Ahmad Hadi</t>
+          <t>Ros Syammimi Bt Hamid</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Yemen</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>A0011223</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2027-05-10</t>
+          <t>2026-12-05</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>+60101234567</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
+          <t>+60134903202</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Faculty Muamalat Pengurusan dan Teknologi</t>
+        </is>
+      </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Software Engineering</t>
+          <t>Bachelor of Information Technology</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -629,106 +633,114 @@
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>201</v>
+        <v>44</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>SAFE</t>
+          <t>URGENT</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 10:28 UTC</t>
+          <t>2026-10-22 14:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>8231123068</t>
+          <t>8231123010</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Abdulrahman Yahaya</t>
+          <t>Ahmad Hadi</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Yemen</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>A122378765</t>
+          <t>A0011223</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr"/>
+          <t>2027-05-10</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>+60101234567</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>FMPT</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineering</t>
+        </is>
+      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>19</v>
+        <v>200</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>SAFE</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 10:28 UTC</t>
+          <t>2026-10-22 14:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>8231123071</t>
+          <t>8231123065</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Abdulrahman yahaya</t>
+          <t>Ahmad Mahram</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Sudan</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>A1122334</t>
+          <t>B0123456</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2027-01-07</t>
+          <t>2027-03-15</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>+601140478950</t>
+          <t>+60325678909</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Computer Science</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -737,54 +749,58 @@
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>78</v>
+        <v>144</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>ACTION_NEEDED</t>
+          <t>SAFE</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 10:28 UTC</t>
+          <t>2026-10-22 14:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>8231123072</t>
+          <t>8231123068</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Usman Usman</t>
+          <t>Abdulrahman Yahaya</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Cameroon</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>A2233445</t>
+          <t>A122378765</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-12-08</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>+60123456789</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>FMPT</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -793,54 +809,58 @@
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>48</v>
+        <v>18</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>URGENT</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 10:28 UTC</t>
+          <t>2026-10-22 14:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>8231123073</t>
+          <t>8231123071</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Muhammad Doshiro</t>
+          <t>Abdulrahman yahaya</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Sudan</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>A3344556</t>
+          <t>A1122334</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-11-08</t>
+          <t>2027-01-07</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>+60134567890</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr"/>
+          <t>+601140478950</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Software Engineering</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -849,51 +869,55 @@
         </is>
       </c>
       <c r="J7" s="2" t="n">
-        <v>18</v>
+        <v>77</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>ACTION_NEEDED</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 10:28 UTC</t>
+          <t>2026-10-22 14:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>8231123074</t>
+          <t>8231123072</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Aminu Ibrahim</t>
+          <t>Usman Usman</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Cameroon</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>A4455667</t>
+          <t>A2233445</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-12-08</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>+60145678901</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
+          <t>+60123456789</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Computer Science</t>
@@ -905,54 +929,58 @@
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>URGENT</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 10:28 UTC</t>
+          <t>2026-10-22 14:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>8231123075</t>
+          <t>8231123073</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Muhammad Mataxuh</t>
+          <t>Muhammad Doshiro</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Chad</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>A5566778</t>
+          <t>A3344556</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2027-02-11</t>
+          <t>2026-11-08</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>+60167890123</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
+          <t>+60134567890</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Software Engineering</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -961,51 +989,55 @@
         </is>
       </c>
       <c r="J9" s="2" t="n">
-        <v>113</v>
+        <v>17</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>SAFE</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 10:28 UTC</t>
+          <t>2026-10-22 14:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>8231123076</t>
+          <t>8231123074</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Muhammad Abdullahi</t>
+          <t>Aminu Ibrahim</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Cote d'Ivoire</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>A6677889</t>
+          <t>A4455667</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2027-03-15</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>+60167890123</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
+          <t>+60145678901</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Computer Science</t>
@@ -1017,54 +1049,58 @@
         </is>
       </c>
       <c r="J10" s="2" t="n">
-        <v>145</v>
+        <v>7</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>SAFE</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 10:28 UTC</t>
+          <t>2026-10-22 14:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>8231123077</t>
+          <t>8231123075</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Abba Ibrahim</t>
+          <t>Muhammad Mataxuh</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Chad</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>A7788990</t>
+          <t>A5566778</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>2027-01-05</t>
+          <t>2027-02-11</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>+60178901234</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr"/>
+          <t>+60167890123</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Software Engineering</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1073,54 +1109,58 @@
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>76</v>
+        <v>112</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>ACTION_NEEDED</t>
+          <t>SAFE</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 10:28 UTC</t>
+          <t>2026-10-22 14:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>8231123078</t>
+          <t>8231123076</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Syed Muhammad</t>
+          <t>Muhammad Abdullahi</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Cote d'Ivoire</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>A8899001</t>
+          <t>A6677889</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-12-15</t>
+          <t>2027-03-15</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>+60189012345</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr"/>
+          <t>+60167890123</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Computer Science</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1129,54 +1169,58 @@
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>55</v>
+        <v>144</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>URGENT</t>
+          <t>SAFE</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 10:28 UTC</t>
+          <t>2026-10-22 14:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>8231123079</t>
+          <t>8231123077</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Arif Amin bin Aziz</t>
+          <t>Abba Ibrahim</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>A9900112</t>
+          <t>A7788990</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026-11-20</t>
+          <t>2027-01-05</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>+60190123456</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr"/>
+          <t>+60178901234</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>Software Engineering</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1185,58 +1229,58 @@
         </is>
       </c>
       <c r="J13" s="2" t="n">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>ACTION_NEEDED</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 10:28 UTC</t>
+          <t>2026-10-22 14:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>UIS-2023-INT156</t>
+          <t>8231123078</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Tanvir Hossain</t>
+          <t>Syed Muhammad</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>BK0982736</t>
+          <t>A8899001</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2026-12-15</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>+60134441234</t>
+          <t>+60189012345</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Faculty of Computing &amp; Informatics</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Bachelor of Computer Science (Cybersecurity)</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1245,7 +1289,7 @@
         </is>
       </c>
       <c r="J14" s="2" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
@@ -1254,49 +1298,49 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 10:28 UTC</t>
+          <t>2026-10-22 14:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>UIS-2023-INT177</t>
+          <t>8231123079</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Fatoumata Camara</t>
+          <t>Arif Amin bin Aziz</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Gambia</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>GM204918</t>
+          <t>A9900112</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2026-12-09</t>
+          <t>2026-11-20</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>+60185556677</t>
+          <t>+60190123456</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Faculty of Islamic Economics &amp; Business</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Bachelor of Accounting (Information Systems)</t>
+          <t>Computer Science</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1305,76 +1349,196 @@
         </is>
       </c>
       <c r="J15" s="2" t="n">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>URGENT</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 10:28 UTC</t>
+          <t>2026-10-22 14:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>UIS-2023-INT156</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Tanvir Hossain</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Bangladesh</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>BK0982736</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-03</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>+60134441234</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Faculty of Computing &amp; Informatics</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Bachelor of Computer Science (Cybersecurity)</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>URGENT</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:54 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>UIS-2023-INT177</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Fatoumata Camara</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Gambia</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>GM204918</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-09</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>+60185556677</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Faculty of Islamic Economics &amp; Business</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Bachelor of Accounting (Information Systems)</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>URGENT</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:54 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>UIS-2025-INT012</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Abdoulaye Diallo</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Guinea</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>GN392014</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>2027-03-07</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>+60148889900</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Faculty of Shariah &amp; Law</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Bachelor of Islamic Law</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="n">
-        <v>137</v>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>136</v>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>SAFE</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-21 10:28 UTC</t>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:54 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>